<commit_message>
docs(tracker): DEFER Epic 6 (Enterprise RBAC) -> future Enterprise Expansion phase
Founder call: DecisionOS is SME-first (owner-run Indian SMEs, ~5-30 people, usually
single-location, phone/OTP-first). Epic 6 (branches, user groups, SSO, per-user API
keys, client portal) solves enterprise/scale problems this segment doesn't have -- and
the existing RBAC (15 granular perms, custom roles, per-user overrides, owner-exclusions,
multi-tenant memberships) already exceeds SME needs. Not a product gap; a segment not
sold to yet. All 5 items -> Deferred; revisit when multi-location / 50+ seat customers land.
NOTE: RBAC-30 (client portal) is really customer-transparency, not RBAC -- revisit under a
'customer engagement' theme with demand validation. Epic 6 is off the SME-launch path.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic6_Enterprise_RBAC.xlsx
+++ b/docs/DecisionOS_Epic6_Enterprise_RBAC.xlsx
@@ -565,17 +565,18 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Multi-location + groups + SSO + API keys + client portal. Post-launch scaling. Kickoff: 2026-08-16.</t>
+          <t>Multi-location + groups + SSO + API keys + client portal. DEFERRED to a future Enterprise Expansion phase -- DecisionOS is SME-first (phone/OTP, single-location, small teams) and the existing RBAC already exceeds SME needs. Revisit when enterprise/multi-location customers land.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Epic 6 progress: 0 of 5 items Done  (0%)</t>
-        </is>
-      </c>
-    </row>
+          <t>Epic 6 DEFERRED -&gt; Enterprise Expansion (future scope). 0 of 5 built; not on the SME-launch path.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
@@ -637,7 +638,7 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Deferred</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -670,7 +671,7 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Deferred</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -703,7 +704,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Deferred</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -1139,7 +1140,7 @@
       </c>
       <c r="I2" s="17" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Deferred</t>
         </is>
       </c>
       <c r="J2" s="16" t="inlineStr"/>
@@ -1193,7 +1194,7 @@
       </c>
       <c r="I3" s="17" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Deferred</t>
         </is>
       </c>
       <c r="J3" s="18" t="inlineStr"/>
@@ -1247,7 +1248,7 @@
       </c>
       <c r="I4" s="17" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Deferred</t>
         </is>
       </c>
       <c r="J4" s="16" t="inlineStr"/>
@@ -1301,7 +1302,7 @@
       </c>
       <c r="I5" s="17" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Deferred</t>
         </is>
       </c>
       <c r="J5" s="18" t="inlineStr"/>
@@ -1355,7 +1356,7 @@
       </c>
       <c r="I6" s="17" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Deferred</t>
         </is>
       </c>
       <c r="J6" s="16" t="inlineStr"/>

</xml_diff>